<commit_message>
Horse herd calc. done assuming no slaughter
</commit_message>
<xml_diff>
--- a/data/prod_parameters/HorseHerd.xlsx
+++ b/data/prod_parameters/HorseHerd.xlsx
@@ -7,7 +7,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="default" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,10 +18,96 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+  <si>
+    <t>f_breed</t>
+  </si>
+  <si>
+    <t>f_prod_system</t>
+  </si>
+  <si>
+    <t>f_animal</t>
+  </si>
+  <si>
+    <t>ponies and Icelandic horses</t>
+  </si>
+  <si>
+    <t>broodmares</t>
+  </si>
+  <si>
+    <t>young horses</t>
+  </si>
+  <si>
+    <t>cold blooded horses</t>
+  </si>
+  <si>
+    <t>riding horses</t>
+  </si>
+  <si>
+    <t>trotters and racehorses</t>
+  </si>
+  <si>
+    <t>low-performing horses</t>
+  </si>
+  <si>
+    <t>medium-performing horses</t>
+  </si>
+  <si>
+    <t>parameter</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>share_of_horses</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>slaughter_weight</t>
+  </si>
+  <si>
+    <t>kg CW</t>
+  </si>
+  <si>
+    <t>live_weight</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -49,8 +135,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -331,9 +421,176 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="2">
+        <v>60.549226441631497</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2">
+        <v>27.5045007032349</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="2">
+        <v>3.7389592123769302</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2">
+        <v>8.2073136427566808</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="2">
+        <v>394.61241132208016</v>
+      </c>
+      <c r="F9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="2">
+        <v>585.45178524024413</v>
+      </c>
+      <c r="F10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="2">
+        <v>567.18533165122039</v>
+      </c>
+      <c r="F11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="2">
+        <v>496.52359083562101</v>
+      </c>
+      <c r="F12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>